<commit_message>
Update Excel layout and UI table to include Channel, Seller Name, Return Date, MP Date, and Days Left columns
</commit_message>
<xml_diff>
--- a/backend/static/sample_upload.xlsx
+++ b/backend/static/sample_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,29 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +62,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,114 +438,250 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Seller Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Return Date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MP Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Days Left</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Invoice No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>AWB</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Courier</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Platform Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>BrandCentral</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>15-09-2026</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>12-09-2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>INV-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>195042600200336</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Delhivery</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Shipped</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Flipkart</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>BrandCentral</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>14-09-2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>11-09-2026</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>INV-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>195042600200337</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Xpressbees</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>In Transit</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Meesho</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>BrandCentral</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>13-09-2026</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>10-09-2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>INV-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>987654321</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Blue Dart</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Myntra</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>BrandCentral</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>12-09-2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>09-09-2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>INV-004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>554433221</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>554483221</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>DTDC</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>

</xml_diff>

<commit_message>
feat: add Order id column after Invoice No. in Sample Excel, upload parser, UI table, and Excel export
</commit_message>
<xml_diff>
--- a/backend/static/sample_upload.xlsx
+++ b/backend/static/sample_upload.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample Upload" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,12 +28,8 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E293B"/>
+      <color rgb="000F172A"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,16 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,18 +428,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,208 +471,181 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Invoice No</t>
+          <t>Invoice No.</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>AWB</t>
+          <t>Order id</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Courier</t>
+          <t>AWB No.</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Courier Partner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Platform Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>BrandCentral</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>12-09-2026</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Meesho</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Brand Central</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>INV-001</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>195042600200336</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Delhivery</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Shipped</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>INV-1001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ORD-982341</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>14345921614930</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Xpressbees</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Return In Transit</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Flipkart</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>BrandCentral</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>14-09-2026</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>11-09-2026</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Brand Central</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>INV-002</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>195042600200337</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Xpressbees</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>In Transit</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>INV-1002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ORD-982342</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>90282192341</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Blue Dart</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Out for Delivery</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>BrandCentral</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>13-09-2026</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>10-09-2026</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Brand Central</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>INV-003</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>987654321</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Blue Dart</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>BrandCentral</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>12-09-2026</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>09-09-2026</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>INV-004</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>554483221</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>DTDC</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>INV-1003</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ORD-982343</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>FMPP1234567890</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ekart</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>

</xml_diff>

<commit_message>
feat: add Item SKU and Amt columns after Order id and add trailing blank columns (Ticket no, Dispute Reason, Remark) in Excel export
</commit_message>
<xml_diff>
--- a/backend/static/sample_upload.xlsx
+++ b/backend/static/sample_upload.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -438,9 +438,11 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,15 +483,25 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Item SKU</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Amt</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>AWB No.</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Courier Partner</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Platform Status</t>
         </is>
@@ -533,15 +545,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>SKU-BC-101</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>499</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>14345921614930</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Xpressbees</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Return In Transit</t>
         </is>
@@ -585,15 +607,25 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>SKU-BC-102</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>799</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>90282192341</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Blue Dart</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Out for Delivery</t>
         </is>
@@ -637,15 +669,25 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>SKU-BC-103</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>FMPP1234567890</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Ekart</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>

</xml_diff>

<commit_message>
feat: add Return Id next to Return Date and Ticket Status in Excel export
</commit_message>
<xml_diff>
--- a/backend/static/sample_upload.xlsx
+++ b/backend/static/sample_upload.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,10 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -58,11 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,21 +433,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,231 +469,251 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Return Id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>MP Date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Days Left</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Invoice No.</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Order id</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Item SKU</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Amt</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AWB No.</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Courier Partner</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Platform Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Meesho</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Brand Central</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>RET-5501</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>INV-1001</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>ORD-982341</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>SKU-BC-101</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>499</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>14345921614930</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Xpressbees</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Return In Transit</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Flipkart</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Brand Central</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>RET-5502</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>INV-1002</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>ORD-982342</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>SKU-BC-102</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>799</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>90282192341</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Blue Dart</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Out for Delivery</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Brand Central</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>RET-5503</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>INV-1003</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>ORD-982343</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>SKU-BC-103</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>FMPP1234567890</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Ekart</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>

</xml_diff>